<commit_message>
working with some mistakes, more din elements nameable
</commit_message>
<xml_diff>
--- a/data/processed/docs_export.xlsx
+++ b/data/processed/docs_export.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>120 01- Kabelzugwinde KZW10.pdf</t>
+          <t>120 01- Kabelzugwinde KZW10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -512,7 +512,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>120 01- Kabelzugwinde KZW10.pdf</t>
+          <t>120 01- Kabelzugwinde KZW10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,7 +551,7 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>120 12- Kettenschutz unten.pdf</t>
+          <t>120 12- Kettenschutz unten</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -590,7 +590,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>120 12- Kettenschutz unten.pdf</t>
+          <t>120 12- Kettenschutz unten</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -629,7 +629,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>120 05- Exzenternabe.pdf</t>
+          <t>120 05- Exzenternabe</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -668,7 +668,7 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>120 06- Distanzscheibe Rastbolzen.pdf</t>
+          <t>120 06- Distanzscheibe Rastbolzen</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -707,7 +707,7 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>120 01 17- Achslager.pdf</t>
+          <t>120 01 17- Achslager</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -739,14 +739,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>61.02.0259</t>
+          <t>61.02.0109</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>120 08 01- Baugrp  Hydraulikmotor.pdf</t>
+          <t>120 01 18- Abschlussblech</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/120 08 01- Baugrp  Hydraulikmotor.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 18- Abschlussblech.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -778,14 +778,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>61.02.0058</t>
+          <t>61.02.0111</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>120 08 02- Kettenrad Z19.pdf</t>
+          <t>120 01 22- Stützplatte</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/120 08 02- Kettenrad Z19.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 22- Stützplatte.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -817,14 +817,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>61.02.0241</t>
+          <t>61.02.0115</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>120 0801 01- Baugrp Konsole Hydromotor.pdf</t>
+          <t>120 01 27- Quertraverse vorne</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 01- Baugrp Konsole Hydromotor.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 27- Quertraverse vorne.pdf</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -856,14 +856,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>61.02.0237</t>
+          <t>61.02.0118</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>120 0801 02- Grundplatte Hydromotor.pdf</t>
+          <t>120 01 30- Gewindehülse M16x40</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 02- Grundplatte Hydromotor.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 30- Gewindehülse M16x40.pdf</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -895,14 +895,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>61.02.0239</t>
+          <t>61.02.0119</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>120 0801 03- Aufnahmeplatte Hydromotor.pdf</t>
+          <t>120 01 31- Gewindehülse M12x40</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 03- Aufnahmeplatte Hydromotor.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 31- Gewindehülse M12x40.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -934,14 +934,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>61.02.0238</t>
+          <t>61.02.0120</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>120 0801 04- Spickel.pdf</t>
+          <t>120 01 32- Gewindehülse M10x40</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 04- Spickel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 32- Gewindehülse M10x40.pdf</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -973,14 +973,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>61.02.0240</t>
+          <t>61.02.0121</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>120 0801 05- Spannkörper.pdf</t>
+          <t>120 01 33- Verankerungslasche hinten</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 05- Spannkörper.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 33- Verankerungslasche hinten.pdf</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1012,14 +1012,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>61.02.0277</t>
+          <t>61.02.0122</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>120 09 01- Baugrp Zugeinheit.pdf</t>
+          <t>120 01 34- Stützenführung</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 01- Baugrp Zugeinheit.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 34- Stützenführung.pdf</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1051,14 +1051,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>61.02.0052</t>
+          <t>61.02.0123</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>120 09 08- Mitnehmerbolzen.pdf</t>
+          <t>120 01 36- Stützenführung vorne</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 08- Mitnehmerbolzen.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 36- Stützenführung vorne.pdf</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1090,14 +1090,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>61.02.0043</t>
+          <t>61.02.0125</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>120 09 05- Spillwelle.pdf</t>
+          <t>120 01 38- Hebeblechlasche</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 05- Spillwelle.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 38- Hebeblechlasche.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1129,14 +1129,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>61.02.0053</t>
+          <t>61.02.0124</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>120 09 19- Wellenschutz.pdf</t>
+          <t>120 01 41- Deichselhalter</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 19- Wellenschutz.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 41- Deichselhalter.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1168,14 +1168,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>61.02.0042</t>
+          <t>61.02.0208</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>120 09 04- Lagerbock.pdf</t>
+          <t>120 01 40- Hebelasche rechts</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 04- Lagerbock.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 40- Hebelasche rechts.pdf</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1207,14 +1207,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>61.02.0230</t>
+          <t>61.02.0299</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>120 09 03- Gegenplatte Lagerbock.pdf</t>
+          <t>120 01 61- Hebelasche</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 03- Gegenplatte Lagerbock.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/01 Baugrp Chassis/120 01 61- Hebelasche.pdf</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1246,14 +1246,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>40.10.7707</t>
+          <t>61.02.0176</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>120 09 02- Grundplatte Lagerbock.pdf</t>
+          <t>120 07 01- Baugrp Rad Ø350</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 02- Grundplatte Lagerbock.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/07 Baugrp Rad/120 07 01- Baugrp Rad Ø350.pdf</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1285,14 +1285,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>61.02.0126</t>
+          <t>61.02.0034</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>120 10 01- Baugrp Seilführungsarm PMC14S.pdf</t>
+          <t>120 07 02- Radachse</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 01- Baugrp Seilführungsarm PMC14S.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/07 Baugrp Rad/120 07 02- Radachse.pdf</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1324,14 +1324,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>61.02.0144</t>
+          <t>61.02.0259</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>120 1004 01- Baugrp Schutz Längenmessung.pdf</t>
+          <t>120 08 01- Baugrp  Hydraulikmotor</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/04 Baugrp Schutz Längenmessung/120 1004 01- Baugrp Schutz Längenmessung.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/120 08 01- Baugrp  Hydraulikmotor.pdf</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1363,14 +1363,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>61.02.0145</t>
+          <t>61.02.0030</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>120 1004 02- Schutzblech hinten.pdf</t>
+          <t>120 08 03- Umlemkachse</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/04 Baugrp Schutz Längenmessung/120 1004 02- Schutzblech hinten.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/120 08 03- Umlemkachse.pdf</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1402,14 +1402,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>61.02.0146</t>
+          <t>61.02.0058</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>120 1004 03- Schutzblech vorne.pdf</t>
+          <t>120 08 02- Kettenrad Z19</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/04 Baugrp Schutz Längenmessung/120 1004 03- Schutzblech vorne.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/120 08 02- Kettenrad Z19.pdf</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1441,14 +1441,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>61.02.0141</t>
+          <t>61.02.0241</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>120 1003 01- Baugrp Schutzrohr.pdf</t>
+          <t>120 0801 01- Baugrp Konsole Hydromotor</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/03 Baugrp Schutzrohr/120 1003 01- Baugrp Schutzrohr.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 01- Baugrp Konsole Hydromotor.pdf</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1480,14 +1480,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>61.02.0142</t>
+          <t>61.02.0237</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>120 1003 02- Schutzrohr.pdf</t>
+          <t>120 0801 02- Grundplatte Hydromotor</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/03 Baugrp Schutzrohr/120 1003 02- Schutzrohr.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 02- Grundplatte Hydromotor.pdf</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1519,14 +1519,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>61.02.0143</t>
+          <t>61.02.0239</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>120 1003 03- Lasche.pdf</t>
+          <t>120 0801 03- Aufnahmeplatte Hydromotor</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/03 Baugrp Schutzrohr/120 1003 03- Lasche.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 03- Aufnahmeplatte Hydromotor.pdf</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1558,14 +1558,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>61.02.0136</t>
+          <t>61.02.0238</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>120 1002 01- Baugrp Support Seilführungsarm.pdf</t>
+          <t>120 0801 04- Spickel</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 01- Baugrp Support Seilführungsarm.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 04- Spickel.pdf</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1597,14 +1597,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>61.02.0137</t>
+          <t>61.02.0240</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>120 1002 02- Grundplatte.pdf</t>
+          <t>120 0801 05- Spannkörper</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 02- Grundplatte.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/08 Baugrp Hydraulikmotor/01 Baugrp Konsole Hydromotor/120 0801 05- Spannkörper.pdf</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1636,14 +1636,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>61.02.0138</t>
+          <t>61.02.0277</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>120 1002 03- Platte hinten.pdf</t>
+          <t>120 09 01- Baugrp Zugeinheit</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 03- Platte hinten.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 01- Baugrp Zugeinheit.pdf</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1675,14 +1675,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>61.02.0139</t>
+          <t>61.02.0052</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>120 1002 04- Spickel.pdf</t>
+          <t>120 09 08- Mitnehmerbolzen</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 04- Spickel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 08- Mitnehmerbolzen.pdf</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1714,14 +1714,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>61.02.0140</t>
+          <t>61.02.0043</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>120 1002 05- Platte vorne.pdf</t>
+          <t>120 09 05- Spillwelle</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 05- Platte vorne.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 05- Spillwelle.pdf</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1753,14 +1753,14 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>61.02.0127</t>
+          <t>61.02.0053</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>120 1001 01- Baugrp Seilführungsarm geschweisst.pdf</t>
+          <t>120 09 19- Wellenschutz</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 01- Baugrp Seilführungsarm geschweisst.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 19- Wellenschutz.pdf</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1792,14 +1792,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>61.02.0128</t>
+          <t>61.02.0042</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>120 1001 09- Längenmessplatte.pdf</t>
+          <t>120 09 04- Lagerbock</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 09- Längenmessplatte.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 04- Lagerbock.pdf</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1831,14 +1831,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>61.02.0129</t>
+          <t>61.02.0230</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>120 1001 08- Seitenteil links.pdf</t>
+          <t>120 09 03- Gegenplatte Lagerbock</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 08- Seitenteil links.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 03- Gegenplatte Lagerbock.pdf</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1870,14 +1870,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>61.02.0130</t>
+          <t>40.10.7707</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>120 1001 07- Seitenteil rechts.pdf</t>
+          <t>120 09 02- Grundplatte Lagerbock</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 07- Seitenteil rechts.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 02- Grundplatte Lagerbock.pdf</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1909,14 +1909,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>61.02.0131</t>
+          <t>61.03.0088</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>120 1001 06- Distanzhalter.pdf</t>
+          <t>018 13 01- Baugrp Haspelachse</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 06- Distanzhalter.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/018 KZW 20/13 Baugrp Haspelachse/018 13 01- Baugrp Haspelachse.pdf</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1948,14 +1948,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>61.02.0132</t>
+          <t>61.03.0138</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>120 1001 05- Lagergehäuse Seilführungsarm.pdf</t>
+          <t>018 13 04- Distanzring</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 05- Lagergehäuse Seilführungsarm.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/018 KZW 20/13 Baugrp Haspelachse/018 13 04- Distanzring.pdf</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1987,14 +1987,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>61.02.0133</t>
+          <t>61.03.0139</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>120 1001 04- Lagerauge.pdf</t>
+          <t>018 13 03- Lageraufnahme</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 04- Lagerauge.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/018 KZW 20/13 Baugrp Haspelachse/018 13 03- Lageraufnahme.pdf</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2026,14 +2026,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>61.02.0134</t>
+          <t>61.03.0137</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>120 1001 03- Zapfenführung.pdf</t>
+          <t>018 13 02- Haspelachse</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 03- Zapfenführung.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/018 KZW 20/13 Baugrp Haspelachse/018 13 02- Haspelachse.pdf</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2065,14 +2065,14 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>61.02.0135</t>
+          <t>61.02.0126</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>120 1001 02- Führungsrohr.pdf</t>
+          <t>120 10 01- Baugrp Seilführungsarm PMC14S</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 02- Führungsrohr.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 01- Baugrp Seilführungsarm PMC14S.pdf</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2104,14 +2104,14 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>61.02.0147</t>
+          <t>61.02.0144</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>120 10 13- Verdrehsicherung.pdf</t>
+          <t>120 1004 01- Baugrp Schutz Längenmessung</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 13- Verdrehsicherung.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/04 Baugrp Schutz Längenmessung/120 1004 01- Baugrp Schutz Längenmessung.pdf</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2143,14 +2143,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>61.02.0148</t>
+          <t>61.02.0145</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>120 10 12- Kraftmesshülse.pdf</t>
+          <t>120 1004 02- Schutzblech hinten</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 12- Kraftmesshülse.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/04 Baugrp Schutz Längenmessung/120 1004 02- Schutzblech hinten.pdf</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2182,14 +2182,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>61.02.0151</t>
+          <t>61.02.0146</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>120 10 09- Hebel.pdf</t>
+          <t>120 1004 03- Schutzblech vorne</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 09- Hebel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/04 Baugrp Schutz Längenmessung/120 1004 03- Schutzblech vorne.pdf</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2221,14 +2221,14 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>61.02.0152</t>
+          <t>61.02.0141</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>120 10 08- Druckstift.pdf</t>
+          <t>120 1003 01- Baugrp Schutzrohr</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 08- Druckstift.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/03 Baugrp Schutzrohr/120 1003 01- Baugrp Schutzrohr.pdf</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2260,14 +2260,14 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>61.02.0154</t>
+          <t>61.02.0142</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>120 10 06- Umlenkhülse.pdf</t>
+          <t>120 1003 02- Schutzrohr</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 06- Umlenkhülse.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/03 Baugrp Schutzrohr/120 1003 02- Schutzrohr.pdf</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2299,14 +2299,14 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>61.02.0155</t>
+          <t>61.02.0143</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>120 10 04- Achse.pdf</t>
+          <t>120 1003 03- Lasche</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 04- Achse.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/03 Baugrp Schutzrohr/120 1003 03- Lasche.pdf</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2338,14 +2338,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>61.02.0156</t>
+          <t>61.02.0136</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>120 10 03- Distanzscheibe.pdf</t>
+          <t>120 1002 01- Baugrp Support Seilführungsarm</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 03- Distanzscheibe.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 01- Baugrp Support Seilführungsarm.pdf</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2377,14 +2377,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>61.02.0157</t>
+          <t>61.02.0137</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>120 10 02- Scheibe.pdf</t>
+          <t>120 1002 02- Grundplatte</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 02- Scheibe.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 02- Grundplatte.pdf</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2416,14 +2416,14 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>61.02.0190</t>
+          <t>61.02.0138</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>120 1201 02- Grundblech.pdf</t>
+          <t>120 1002 03- Platte hinten</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/12 Baugrp Seileinlauf/01 Baugrp Seileinlauf geschweisst/120 1201 02- Grundblech.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 03- Platte hinten.pdf</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2455,14 +2455,14 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>61.02.0182</t>
+          <t>61.02.0139</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>120 16 01- Baugrp Hebeblech.pdf</t>
+          <t>120 1002 04- Spickel</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 01- Baugrp Hebeblech.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 04- Spickel.pdf</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2494,14 +2494,14 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>61.02.0183</t>
+          <t>61.02.0140</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>120 16 02- Hebeblech.pdf</t>
+          <t>120 1002 05- Platte vorne</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 02- Hebeblech.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/02 Baugrp Support Seilführungsarm/120 1002 05- Platte vorne.pdf</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2533,14 +2533,14 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>61.02.0184</t>
+          <t>61.02.0127</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>120 16 06- Auflage Hebeblech.pdf</t>
+          <t>120 1001 01- Baugrp Seilführungsarm geschweisst</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 06- Auflage Hebeblech.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 01- Baugrp Seilführungsarm geschweisst.pdf</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2572,14 +2572,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>61.02.0228</t>
+          <t>61.02.0128</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>120 16 11- Baugrp Verstellhebel Hebeblech.pdf</t>
+          <t>120 1001 09- Längenmessplatte</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 11- Baugrp Verstellhebel Hebeblech.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 09- Längenmessplatte.pdf</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2611,14 +2611,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>61.02.0226</t>
+          <t>61.02.0129</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>120 16 12- Verstellwelle.pdf</t>
+          <t>120 1001 08- Seitenteil links</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 12- Verstellwelle.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 08- Seitenteil links.pdf</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2650,14 +2650,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>61.02.0227</t>
+          <t>61.02.0130</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>120 16 13- Verstellhebel.pdf</t>
+          <t>120 1001 07- Seitenteil rechts</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 13- Verstellhebel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 07- Seitenteil rechts.pdf</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2689,14 +2689,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>61.02.0278</t>
+          <t>61.02.0131</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>120 17 03- Baugrp Bremselement geschweisst.pdf</t>
+          <t>120 1001 06- Distanzhalter</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 03- Baugrp Bremselement geschweisst.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 06- Distanzhalter.pdf</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2728,14 +2728,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>61.02.0251</t>
+          <t>61.02.0132</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>120 17 11- Seitenteil Haspelbremse.pdf</t>
+          <t>120 1001 05- Lagergehäuse Seilführungsarm</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 11- Seitenteil Haspelbremse.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 05- Lagergehäuse Seilführungsarm.pdf</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2767,14 +2767,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>61.02.0251-L</t>
+          <t>61.02.0133</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>120 17 11- Seitenteil Haspelbremse.pdf</t>
+          <t>120 1001 04- Lagerauge</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 11- Seitenteil Haspelbremse.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 04- Lagerauge.pdf</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2806,14 +2806,14 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>40.10.3065</t>
+          <t>61.02.0134</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>120 17 13- Rohr.pdf</t>
+          <t>120 1001 03- Zapfenführung</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 13- Rohr.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 03- Zapfenführung.pdf</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2845,14 +2845,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>40.10.2113</t>
+          <t>61.02.0135</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>120 17 14- Segment.pdf</t>
+          <t>120 1001 02- Führungsrohr</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 14- Segment.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/01 Baugrp Seilführungsarm geschweisst/120 1001 02- Führungsrohr.pdf</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2884,14 +2884,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>61.03.0077</t>
+          <t>61.02.0147</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>120 17 02- Baugrp Bremshebel.pdf</t>
+          <t>120 10 13- Verdrehsicherung</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 02- Baugrp Bremshebel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 13- Verdrehsicherung.pdf</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2923,14 +2923,14 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>40.10.7481</t>
+          <t>61.02.0148</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>120 17 12- Federhalter.pdf</t>
+          <t>120 10 12- Kraftmesshülse</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 12- Federhalter.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 12- Kraftmesshülse.pdf</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2962,14 +2962,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>61.03.0188</t>
+          <t>61.02.0149</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>120 17 15- Bremshebel.pdf</t>
+          <t>120 10 11- Kraftmessrolle</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 15- Bremshebel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 11- Kraftmessrolle.pdf</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3001,14 +3001,14 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>61.03.0189</t>
+          <t>61.02.0150</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>120 17 16- Nabe Bremshebel.pdf</t>
+          <t>120 10 10- Längenmessrolle</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 16- Nabe Bremshebel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 10- Längenmessrolle.pdf</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3040,14 +3040,14 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>61.02.0158</t>
+          <t>61.02.0151</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
-          <t>120 22 01- Baugrp Abstützung vorn.pdf</t>
+          <t>120 10 09- Hebel</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/22 Baugrp Abstützung vorn/120 22 01- Baugrp Abstützung vorn.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 09- Hebel.pdf</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3079,14 +3079,14 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>61.02.0159</t>
+          <t>61.02.0152</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>120 22 02- Hohlprofil 30x30x2.5 DIN EN 10305-5.pdf</t>
+          <t>120 10 08- Druckstift</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/22 Baugrp Abstützung vorn/120 22 02- Hohlprofil 30x30x2.5 DIN EN 10305-5.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 08- Druckstift.pdf</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3118,14 +3118,14 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>61.02.0160</t>
+          <t>61.02.0154</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>120 23 03- Stützplatte.pdf</t>
+          <t>120 10 06- Umlenkhülse</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/23 Baugrp Abstützung/120 23 03- Stützplatte.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 06- Umlenkhülse.pdf</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3157,14 +3157,14 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>61.02.0161</t>
+          <t>61.02.0155</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>120 23 01- Baugrp Abstützung.pdf</t>
+          <t>120 10 04- Achse</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/23 Baugrp Abstützung/120 23 01- Baugrp Abstützung.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 04- Achse.pdf</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3196,14 +3196,14 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>61.02.0162</t>
+          <t>61.02.0156</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
-          <t>120 23 02- Hohlprofil 30x30x2.5 DIN EN 10305-5.pdf</t>
+          <t>120 10 03- Distanzscheibe</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/23 Baugrp Abstützung/120 23 02- Hohlprofil 30x30x2.5 DIN EN 10305-5.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 03- Distanzscheibe.pdf</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3235,14 +3235,14 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>61.02.0222</t>
+          <t>61.02.0157</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>120 26 11- Befestigungsrohr.pdf</t>
+          <t>120 10 02- Scheibe</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/26 Baugrp Deichsel/120 26 11- Befestigungsrohr.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/10 Baugrp Seilführungsarm/120 10 02- Scheibe.pdf</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3274,14 +3274,14 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>61.02.0224</t>
+          <t>61.02.0199</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
-          <t>120 26 13- Deichselrohr.pdf</t>
+          <t>120 12 01- Baugrp Seileinlauf</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/26 Baugrp Deichsel/120 26 13- Deichselrohr.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/12 Baugrp Seileinlauf/120 12 01- Baugrp Seileinlauf.pdf</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3313,14 +3313,14 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>61.02.0212</t>
+          <t>61.02.0195</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>120 0506 23- Träger BM.pdf</t>
+          <t>120 12 02- Rolle Seileinlauf</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/06 Baugrp Hydrauliktank/120 0506 23- Träger BM.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/12 Baugrp Seileinlauf/120 12 02- Rolle Seileinlauf.pdf</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3352,14 +3352,14 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>61.02.0175</t>
+          <t>61.02.0225</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
-          <t>120 0505 17- Pumpenanlenkung.pdf</t>
+          <t>120 12 03- Achse Seileinlauf</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 17- Pumpenanlenkung.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/12 Baugrp Seileinlauf/120 12 03- Achse Seileinlauf.pdf</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3391,14 +3391,14 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>61.02.0250</t>
+          <t>61.02.0189</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
-          <t>120 24 05- Stecknagel.pdf</t>
+          <t>120 12 06- Seileinlauf oben</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 05- Stecknagel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/12 Baugrp Seileinlauf/120 12 06- Seileinlauf oben.pdf</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3430,14 +3430,14 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>61.02.0249</t>
+          <t>61.02.0194</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>120 02- Gegenplatte Halter Haspelachse.pdf</t>
+          <t>120 1201 01- Baugrp Seileinlauf geschweisst</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/120 02- Gegenplatte Halter Haspelachse.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/12 Baugrp Seileinlauf/01 Baugrp Seileinlauf geschweisst/120 1201 01- Baugrp Seileinlauf geschweisst.pdf</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3469,14 +3469,14 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>61.02.0245</t>
+          <t>61.02.0190</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>120 24 01- Baugrp Halter Haspelachse.pdf</t>
+          <t>120 1201 02- Grundblech</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 01- Baugrp Halter Haspelachse.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/12 Baugrp Seileinlauf/01 Baugrp Seileinlauf geschweisst/120 1201 02- Grundblech.pdf</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3508,14 +3508,14 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>61.02.0242</t>
+          <t>61.02.0182</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
-          <t>120 24 02- Grundplatte.pdf</t>
+          <t>120 16 01- Baugrp Hebeblech</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 02- Grundplatte.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 01- Baugrp Hebeblech.pdf</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3547,14 +3547,14 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>61.02.0243</t>
+          <t>61.02.0183</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>120 24 03- Spickel.pdf</t>
+          <t>120 16 02- Hebeblech</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 03- Spickel.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 02- Hebeblech.pdf</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3586,14 +3586,14 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>61.02.0279</t>
+          <t>61.02.0184</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>120 09 01- Baugrp Zugeinheit.pdf</t>
+          <t>120 16 06- Auflage Hebeblech</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 01- Baugrp Zugeinheit.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 06- Auflage Hebeblech.pdf</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3625,14 +3625,14 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>61.03.0280</t>
+          <t>61.02.0228</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>120 09 10- Baugrp Spill.pdf</t>
+          <t>120 16 11- Baugrp Verstellhebel Hebeblech</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 10- Baugrp Spill.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 11- Baugrp Verstellhebel Hebeblech.pdf</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3664,14 +3664,14 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>61.03.0099</t>
+          <t>61.02.0226</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>120 09 07- Spill.pdf</t>
+          <t>120 16 12- Verstellwelle</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 07- Spill.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 12- Verstellwelle.pdf</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3703,14 +3703,14 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>61.02.0044</t>
+          <t>61.02.0227</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
-          <t>120 09 06- Spillnabe.pdf</t>
+          <t>120 16 13- Verstellhebel</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 06- Spillnabe.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/16 Baugrp Hebeblech/120 16 13- Verstellhebel.pdf</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3742,14 +3742,14 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>60.02.5110</t>
+          <t>61.02.0278</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>120 33 01-  Baugrp Fernbetätigung Pumpe.pdf</t>
+          <t>120 17 03- Baugrp Bremselement geschweisst</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/33 Baugrp Fernbetätigung Pumpe/120 33 01-  Baugrp Fernbetätigung Pumpe.pdf</t>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 03- Baugrp Bremselement geschweisst.pdf</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3781,14 +3781,14 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>60.02.5115</t>
+          <t>61.02.0251</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
-          <t>120 02 01- Baugrp Messsteuerung PMC14S.pdf</t>
+          <t>120 17 11- Seitenteil Haspelbremse</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3798,20 +3798,2477 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 11- Seitenteil Haspelbremse.pdf</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>61.02.0251-L</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>120 17 11- Seitenteil Haspelbremse</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 11- Seitenteil Haspelbremse.pdf</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>61.03.0078</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>120 17 04- Baugrp Bremselement</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 04- Baugrp Bremselement.pdf</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>40.10.3065</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>120 17 13- Rohr</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 13- Rohr.pdf</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>40.10.2113</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>120 17 14- Segment</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 14- Segment.pdf</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>61.03.0077</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>120 17 02- Baugrp Bremshebel</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 02- Baugrp Bremshebel.pdf</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>40.10.7481</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>120 17 12- Federhalter</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 12- Federhalter.pdf</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>61.03.0188</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>120 17 15- Bremshebel</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 15- Bremshebel.pdf</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>61.03.0189</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>120 17 16- Nabe Bremshebel</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/17 Baugrp Haspelbremse/120 17 16- Nabe Bremshebel.pdf</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>61.02.0158</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>120 22 01- Baugrp Abstützung vorn</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/22 Baugrp Abstützung vorn/120 22 01- Baugrp Abstützung vorn.pdf</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>61.02.0159</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>120 22 02- Hohlprofil 30x30x2.5 DIN EN 10305-5</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/22 Baugrp Abstützung vorn/120 22 02- Hohlprofil 30x30x2.5 DIN EN 10305-5.pdf</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>61.02.0160</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>120 23 03- Stützplatte</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/23 Baugrp Abstützung/120 23 03- Stützplatte.pdf</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>61.02.0161</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>120 23 01- Baugrp Abstützung</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/23 Baugrp Abstützung/120 23 01- Baugrp Abstützung.pdf</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>61.02.0162</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr"/>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>120 23 02- Hohlprofil 30x30x2.5 DIN EN 10305-5</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/23 Baugrp Abstützung/120 23 02- Hohlprofil 30x30x2.5 DIN EN 10305-5.pdf</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>61.02.0222</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>120 26 11- Befestigungsrohr</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/26 Baugrp Deichsel/120 26 11- Befestigungsrohr.pdf</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>61.02.0224</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>120 26 13- Deichselrohr</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/26 Baugrp Deichsel/120 26 13- Deichselrohr.pdf</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>61.02.0164</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr"/>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>120 0506 11- Pumpenträger</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/06 Baugrp Hydrauliktank/120 0506 11- Pumpenträger.pdf</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>61.02.0165</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr"/>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>120 0506 12- Grundblech</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/06 Baugrp Hydrauliktank/120 0506 12- Grundblech.pdf</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>61.02.0168</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>120 0506 15- Einschweissbuchse M8</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/06 Baugrp Hydrauliktank/120 0506 15- Einschweissbuchse M8.pdf</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>61.02.0170</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr"/>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>120 0506 17- Anschweissbuchse 3_4</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/06 Baugrp Hydrauliktank/120 0506 17- Anschweissbuchse 3_4.pdf</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>61.02.0172</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr"/>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>120 0506 21- Anschweissbuchse 3_8 lang</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/06 Baugrp Hydrauliktank/120 0506 21- Anschweissbuchse 3_8 lang.pdf</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>61.02.0212</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>120 0506 23- Träger BM</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/06 Baugrp Hydrauliktank/120 0506 23- Träger BM.pdf</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>61.02.0213</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr"/>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>120 0505 06- Baugrp Pumpenhebel</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 06- Baugrp Pumpenhebel.pdf</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>61.02.0214</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>120 0505 14- Verstellrohr</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 14- Verstellrohr.pdf</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>61.02.0173</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr"/>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>120 0505 05- Baugrp Pumpenanlenkung</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 05- Baugrp Pumpenanlenkung.pdf</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>61.02.0174</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr"/>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>120 0505 16- Anschweisshebel</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 16- Anschweisshebel.pdf</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>61.02.0175</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>120 0505 17- Pumpenanlenkung</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 17- Pumpenanlenkung.pdf</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>61.02.0178</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr"/>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>120 0505 04- Baugrp Pumpenblech</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 04- Baugrp Pumpenblech.pdf</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>61.02.0179</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>120 0505 13- Pumpenblech</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 13- Pumpenblech.pdf</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>61.02.0220</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr"/>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>120 0505 01- Baugrp Hydraulikpumpe</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/05 Baugrp Hydraulikpumpe/120 0505 01- Baugrp Hydraulikpumpe.pdf</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>61.02.0250</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr"/>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>120 24 05- Stecknagel</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 05- Stecknagel.pdf</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>61.02.0249</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr"/>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>120 02- Gegenplatte Halter Haspelachse</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/120 02- Gegenplatte Halter Haspelachse.pdf</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>61.02.0245</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr"/>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>120 24 01- Baugrp Halter Haspelachse</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 01- Baugrp Halter Haspelachse.pdf</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>61.02.0242</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>120 24 02- Grundplatte</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 02- Grundplatte.pdf</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>61.02.0243</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr"/>
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>120 24 03- Spickel</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/24 Baugrp Halter Haspelachse/120 24 03- Spickel.pdf</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>61.02.0219</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr"/>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>120 05 01- Baugrp Power Unit BM+EM</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/120 05 01- Baugrp Power Unit BM+EM.pdf</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>61.02.0216</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr"/>
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>120 05 12- Distanzring Fliehkraftkupplung BM kombi EM</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/120 05 12- Distanzring Fliehkraftkupplung BM kombi EM.pdf</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>61.02.0217</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
+      <c r="C124" t="inlineStr"/>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>120 05 13- Distanzring Kupplung 2R</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/120 05 13- Distanzring Kupplung 2R.pdf</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>61.02.0218</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="inlineStr"/>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>120 05 14- Keilriemen SPA 825</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/120 05 14- Keilriemen SPA 825.pdf</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>61.02.0221</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="inlineStr"/>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>120 0504 01- Baugrp Elektromotor kombiniert</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/05 Baugrp Power Unit/04 Baugrp Elektromotor/120 0504 01- Baugrp Elektromotor kombiniert.pdf</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>60.06.0500</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="inlineStr"/>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>190 05 01- Baugrp Haspel Nr.5</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 01- Baugrp Haspel Nr.5.pdf</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>61.02.0281</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>190 05 18- Querstrebe</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 18- Querstrebe.pdf</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>61.06.0250</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>190 05 15- Rohrreif</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 15- Rohrreif.pdf</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>61.02.0283</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="inlineStr"/>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>190 05 11- Querstrebe</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 11- Querstrebe.pdf</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>61.02.0284</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr"/>
+      <c r="C131" t="inlineStr"/>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>190 05 10- Seitenwand</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 10- Seitenwand.pdf</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>61.02.0288</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>190 05 04- Baugrp Querstrebe verstärkt</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 04- Baugrp Querstrebe verstärkt.pdf</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>61.02.0287</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>190 05 16- Verstärkung</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 16- Verstärkung.pdf</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>61.02.0289</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>190 05 12- Querstrebe</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 12- Querstrebe.pdf</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>61.02.0290</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>190 05 03- Baugrp Haspellager</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 03- Baugrp Haspellager.pdf</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>40.10.8022</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr"/>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>190 05 17- Winkel</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 17- Winkel.pdf</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>61.02.0292</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>190 05 02- Baugrp Haspelrohr mit Seilhaken</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 02- Baugrp Haspelrohr mit Seilhaken.pdf</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>61.02.0291</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr"/>
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>190 05 13- Seilhaken</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 13- Seilhaken.pdf</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>61.02.0293</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>190 05 19- Haspelrohr</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/190 Haspel/190 05- Baugrp Haspel Nr.5/190 05 19- Haspelrohr.pdf</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>61.02.0279</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>120 09 01- Baugrp Zugeinheit</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 01- Baugrp Zugeinheit.pdf</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>61.03.0280</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>120 09 10- Baugrp Spill</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 10- Baugrp Spill.pdf</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>61.03.0099</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr"/>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>120 09 07- Spill</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 07- Spill.pdf</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>61.02.0044</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>120 09 06- Spillnabe</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/09 Baugrp Zugeinheit/120 09 06- Spillnabe.pdf</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>60.02.5110</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>120 33 01-  Baugrp Fernbetätigung Pumpe</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/33 Baugrp Fernbetätigung Pumpe/120 33 01-  Baugrp Fernbetätigung Pumpe.pdf</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>61.02.0209</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr"/>
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>120 02 13- Winkel Bedienung</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/02 Baugrp Messsteuerung PMC14S/120 02 13- Winkel Bedienung.pdf</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>61.02.0211</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>120 02 14- Halter Bedienung</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/02 Baugrp Messsteuerung PMC14S/120 02 14- Halter Bedienung.pdf</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>61.02.0206</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>120 0202 21- Gurthalter</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/02 Baugrp Messsteuerung PMC14S/02 Baugrp Bedieneinheit/120 0202 21- Gurthalter.pdf</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>60.02.5115</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr"/>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>120 02 01- Baugrp Messsteuerung PMC14S</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
           <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/02 Baugrp Messsteuerung PMC14S/120 02 01- Baugrp Messsteuerung PMC14S.pdf</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>12.64.0120</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr"/>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>120 0201 01- Baugrp Klemmenkasten</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/02 Baugrp Messsteuerung PMC14S/01 Baugrp Klemmenkasten/120 0201 01- Baugrp Klemmenkasten.pdf</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>JOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>12.64.0121</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr"/>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>120 0202 01- Baugrp Bedieneinheit</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>T:/01 Jost AG/05 Produktion/11 Eigenprodukte Jost/11 Eigenprodukte Jost/120 KZW 10/02 Baugrp Messsteuerung PMC14S/02 Baugrp Bedieneinheit/120 0202 01- Baugrp Bedieneinheit.pdf</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
         <is>
           <t>JOS</t>
         </is>

</xml_diff>